<commit_message>
Update 10 terms in BCIO_Engagement.xlsx
</commit_message>
<xml_diff>
--- a/Engagement/BCIO_Engagement.xlsx
+++ b/Engagement/BCIO_Engagement.xlsx
@@ -700,81 +700,74 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050521</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>BCI engagement period statistic</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>A data item that is about a collection of BCI engagement periods.</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BCI engagement period</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="n"/>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="n"/>
-      <c r="W4" s="3" t="n"/>
-      <c r="X4" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:013085</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Decreased engagement</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> remove  </t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="n"/>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="n"/>
+      <c r="W4" s="2" t="n"/>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>EJH</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BCIO:013085</t>
+          <t>BCIO:013080</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Decreased engagement</t>
+          <t>Increased engagement</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> remove  </t>
+          <t xml:space="preserve">remove
+</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -795,7 +788,11 @@
           <t>Engagement</t>
         </is>
       </c>
-      <c r="R5" s="2" t="n"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Can we add time related entities? Ontologically correct? Thinking probably best to leave for this version</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -818,20 +815,15 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BCIO:013080</t>
+          <t>BCIO:013090</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Increased engagement</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">remove
-</t>
-        </is>
-      </c>
+          <t>Same engagement</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
@@ -850,11 +842,7 @@
           <t>Engagement</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Can we add time related entities? Ontologically correct? Thinking probably best to leave for this version</t>
-        </is>
-      </c>
+      <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -875,108 +863,120 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:013090</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Same engagement</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="n"/>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="n"/>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>EJH</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:013030</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>aggregate behavioural BCI engagement duration</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>A temporal interval that is the sum of the duration of behavioural BCI engagements for a BCI.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>behavioural BCI engagement</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>A unit of time that describes the summed duration of all BCI engagement events.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>90 minutes total app usage, 12 hours of counselling sessions</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Describes the total duration of engagement in a BCI (e.g., all face-to-face sessions AND all telephone contacts), or the total duration of engagement in part of a BCI (e.g., all face-to-face sessions only). (A unit of time that describes the summed duration of all BCI engagement events.) 
+Depending on how “aggregate BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 50 minutes in total across the sessions, (2) maximum (e.g., participants talked to the therapist for up to 4.5 hours in total across the sessions, (3) mean (e.g., participants talked with the therapist, on average, for 3 hours in total across the sessions) or (4) median (e.g., the median length of time participants talked with therapists in all their session was 3 hours). </t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="n"/>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="n"/>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>EJH; Ai; PS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013030</t>
+          <t>BCIO:050522</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>aggregate behavioural BCI engagement duration statistic</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>A data item that is about a collection of aggregate behavioural BCI engagement durations.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
           <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>A temporal interval that is the sum of the duration of behavioural BCI engagements for a BCI.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>A unit of time that describes the summed duration of all BCI engagement events.</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>90 minutes total app usage, 12 hours of counselling sessions</t>
-        </is>
-      </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
+      <c r="M8" s="3" t="n"/>
       <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Describes the total duration of engagement in a BCI (e.g., all face-to-face sessions AND all telephone contacts), or the total duration of engagement in part of a BCI (e.g., all face-to-face sessions only). (A unit of time that describes the summed duration of all BCI engagement events.) 
-Depending on how “aggregate BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 50 minutes in total across the sessions, (2) maximum (e.g., participants talked to the therapist for up to 4.5 hours in total across the sessions, (3) mean (e.g., participants talked with the therapist, on average, for 3 hours in total across the sessions) or (4) median (e.g., the median length of time participants talked with therapists in all their session was 3 hours). </t>
-        </is>
-      </c>
+      <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -999,161 +999,178 @@
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MF:0000018</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>attending</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A mental process whereby relevant aspects of one's mental experience are focused on specific targets. </t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>mental process</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Focusing on particular internal or external stimuli.</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Ai; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:013010</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>behavioural BCI engagement</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Participant engagement with behaviour change intervention in which the engagement activity is a behaviour. </t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>participant engagement with behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Any behaviour performed to engage with an intervention and its content.</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Eye movements, body movements, meditation, attending an intervention session, using nicotine patches in a smoking cessation intervention, or online activity: attending, logging in, posting on a discussion board, reading content, mouse clicks, viewing, using tools, journaling</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>This is distinguished from engagement that involves thought processes.</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="n"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="n"/>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
           <t>EJH; Ai; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050522</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration statistic</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>A data item that is about a collection of aggregate behavioural BCI engagement durations.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V9" s="3" t="n"/>
-      <c r="W9" s="3" t="n"/>
-      <c r="X9" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MF:0000018</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>attending</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A mental process whereby relevant aspects of one's mental experience are focused on specific targets. </t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>mental process</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Focusing on particular internal or external stimuli.</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>Ai; PS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013010</t>
+          <t>BCIO:013025</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>behavioural BCI engagement duration</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal interval between the start and end of a behavioural BCI engagement. </t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
           <t>behavioural BCI engagement</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Participant engagement with behaviour change intervention in which the engagement activity is a behaviour. </t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>one-dimensional temporal region</t>
         </is>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Any behaviour performed to engage with an intervention and its content.</t>
+          <t>A unit of time that describes the length of an engagement event.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Eye movements, body movements, meditation, attending an intervention session, using nicotine patches in a smoking cessation intervention, or online activity: attending, logging in, posting on a discussion board, reading content, mouse clicks, viewing, using tools, journaling</t>
+          <t>A 30-minute session, 1 hour spent 'logged in'</t>
         </is>
       </c>
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>This is distinguished from engagement that involves thought processes.</t>
+          <t>The class “BCI engagement duration” can be used multiple times to capture the frequency of different types of engagements, such as the frequency of engaging with social media or printed material. 
+Depending on how “BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 10 minutes in each session, (2) maximum (e.g., participants talked to the therapist for up to 1 hour in each session, (3) mean (e.g., participants talked with the therapist for 45 minutes on average in each session) or (4) median (e.g., the median length of calls between participants and therapists was 42 minutes in each session).</t>
         </is>
       </c>
       <c r="P11" s="3" t="n"/>
@@ -1185,17 +1202,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013025</t>
+          <t>BCIO:013020</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement frequency</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A temporal interval between the start and end of a behavioural BCI engagement. </t>
+          <t>A data item that is about the number of times behavioural BCI engagement occurs within a unit of time.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1207,18 +1224,14 @@
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>A unit of time that describes the length of an engagement event.</t>
-        </is>
-      </c>
+      <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>A 30-minute session, 1 hour spent 'logged in'</t>
+          <t xml:space="preserve">Hourly, daily, weekly or monthly encounters. </t>
         </is>
       </c>
       <c r="K12" s="3" t="n"/>
@@ -1231,8 +1244,9 @@
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>The class “BCI engagement duration” can be used multiple times to capture the frequency of different types of engagements, such as the frequency of engaging with social media or printed material. 
-Depending on how “BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 10 minutes in each session, (2) maximum (e.g., participants talked to the therapist for up to 1 hour in each session, (3) mean (e.g., participants talked with the therapist for 45 minutes on average in each session) or (4) median (e.g., the median length of calls between participants and therapists was 42 minutes in each session).</t>
+          <t xml:space="preserve">Describes the frequency of BCI engagement in a BCI (e.g., participants had weekly contact), or the frequency of engagement in part of a BCI (e.g., participants received face-to-face contact once a month). 
+The class “BCI engagement frequency” can be used to capture the frequency of different types of engagement, such as the frequency of engaging with social media or printed material. 
+Depending on how “BCI engagement frequency” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants joined at least 1 session every week), (2) maximum (e.g., only 10% of participants attended 5 sessions every week), (3) mean (e.g., participants joined 4 sessions per week on average) or (4) median (e.g., the median number of sessions participants attended was 4 per week). </t>
         </is>
       </c>
       <c r="P12" s="3" t="n"/>
@@ -1257,29 +1271,29 @@
       <c r="W12" s="3" t="n"/>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050523</t>
+          <t>BCIO:050524</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement frequency statistic</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about a collection of behavioural BCI engagement durations.</t>
+          <t>A data item that is about a collection of behavioural BCI engagement frequencies.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
@@ -1326,17 +1340,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013020</t>
+          <t>BCIO:050525</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency</t>
+          <t>behavioural BCI engagement number statistic</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about the number of times behavioural BCI engagement occurs within a unit of time.</t>
+          <t>A data item that is about a collection of behavioural BCI engagement contact event numbers.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1353,26 +1367,12 @@
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hourly, daily, weekly or monthly encounters. </t>
-        </is>
-      </c>
+      <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
+      <c r="M14" s="3" t="n"/>
       <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Describes the frequency of BCI engagement in a BCI (e.g., participants had weekly contact), or the frequency of engagement in part of a BCI (e.g., participants received face-to-face contact once a month). 
-The class “BCI engagement frequency” can be used to capture the frequency of different types of engagement, such as the frequency of engaging with social media or printed material. 
-Depending on how “BCI engagement frequency” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants joined at least 1 session every week), (2) maximum (e.g., only 10% of participants attended 5 sessions every week), (3) mean (e.g., participants joined 4 sessions per week on average) or (4) median (e.g., the median number of sessions participants attended was 4 per week). </t>
-        </is>
-      </c>
+      <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="inlineStr">
         <is>
@@ -1395,29 +1395,29 @@
       <c r="W14" s="3" t="n"/>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; CM; PS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050524</t>
+          <t>BCIO:050523</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about a collection of behavioural BCI engagement frequencies.</t>
+          <t>A data item that is about a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E15" s="3" t="n"/>
@@ -1464,39 +1464,47 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050525</t>
+          <t>BCIO:013040</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>cognitive BCI engagement</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about a collection of behavioural BCI engagement contact event numbers.</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>behavioural BCI engagement</t>
-        </is>
-      </c>
+          <t>Participant engagement with behaviour change intervention in which the engagement activity is a cognitive process.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>cognitive process</t>
+        </is>
+      </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>participant engagement with behaviour change intervention</t>
         </is>
       </c>
       <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paying attention or understanding an intervention’s content, thinking, forming, or changing beliefs about intervention </t>
+        </is>
+      </c>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
       <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Describes engagement which can be demonstrated through reviewing, understanding, learning or recalling the intervention content. Cognitive processes entail the act of directing the mind to see, listen or understand.</t>
+        </is>
+      </c>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="inlineStr">
         <is>
@@ -1519,52 +1527,56 @@
       <c r="W16" s="3" t="n"/>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013040</t>
+          <t>BCIO:013045</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement</t>
+          <t xml:space="preserve">cognitive BCI engagement through attention </t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Participant engagement with behaviour change intervention in which the engagement activity is a cognitive process.</t>
+          <t>A cognitive BCI engagement that involves attending.</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>cognitive process</t>
+          <t>attending</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>cognitive BCI engagement</t>
         </is>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paying attention or understanding an intervention’s content, thinking, forming, or changing beliefs about intervention </t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="n"/>
+          <t>Paying attention to an intervention’s content</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Paying attention to certain images or information within the intervention</t>
+        </is>
+      </c>
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3" t="n"/>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Describes engagement which can be demonstrated through reviewing, understanding, learning or recalling the intervention content. Cognitive processes entail the act of directing the mind to see, listen or understand.</t>
+          <t>“Attending” is defined as “The process whereby relevant aspects of our mental experience are focused on specific targets.”</t>
         </is>
       </c>
       <c r="P17" s="3" t="n"/>
@@ -1589,31 +1601,31 @@
       <c r="W17" s="3" t="n"/>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; CM; PS</t>
+          <t>EJH; Ai; PS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013045</t>
+          <t>BCIO:013050</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cognitive BCI engagement through attention </t>
+          <t xml:space="preserve">cognitive BCI engagement through comprehension </t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>A cognitive BCI engagement that involves attending.</t>
+          <t>A cognitive BCI engagement that involves comprehension.</t>
         </is>
       </c>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>attending</t>
+          <t>comprehension</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1622,14 +1634,10 @@
         </is>
       </c>
       <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Paying attention to an intervention’s content</t>
-        </is>
-      </c>
+      <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Paying attention to certain images or information within the intervention</t>
+          <t>Comprehension of meaning, requirements or importance. Formal testing, providing feedback</t>
         </is>
       </c>
       <c r="K18" s="3" t="n"/>
@@ -1638,7 +1646,7 @@
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>“Attending” is defined as “The process whereby relevant aspects of our mental experience are focused on specific targets.”</t>
+          <t>“Comprehension” is defined as “A cognitive process that creates a representation of the meaning and significance of a communication, object, event or situation.”</t>
         </is>
       </c>
       <c r="P18" s="3" t="n"/>
@@ -1663,31 +1671,31 @@
       <c r="W18" s="3" t="n"/>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013050</t>
+          <t>BCIO:013055</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cognitive BCI engagement through comprehension </t>
+          <t>cognitive BCI engagement through judging</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>A cognitive BCI engagement that involves comprehension.</t>
+          <t>A cognitive BCI engagement that involves a judging process.</t>
         </is>
       </c>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>comprehension</t>
+          <t>judging</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1696,19 +1704,19 @@
         </is>
       </c>
       <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Comprehension of meaning, requirements or importance. Formal testing, providing feedback</t>
-        </is>
-      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Evaluations of usefulness, relevance usability or effectiveness.</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3" t="n"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>“Comprehension” is defined as “A cognitive process that creates a representation of the meaning and significance of a communication, object, event or situation.”</t>
+          <t>“Judging” is defined as “A &lt;mental process&gt; during which information is evaluated, the outcome of which is a belief or opinion.”</t>
         </is>
       </c>
       <c r="P19" s="3" t="n"/>
@@ -1738,269 +1746,269 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:013055</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>cognitive BCI engagement through judging</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>A cognitive BCI engagement that involves a judging process.</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>judging</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>cognitive BCI engagement</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Evaluations of usefulness, relevance usability or effectiveness.</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>“Judging” is defined as “A &lt;mental process&gt; during which information is evaluated, the outcome of which is a belief or opinion.”</t>
-        </is>
-      </c>
-      <c r="P20" s="3" t="n"/>
-      <c r="Q20" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R20" s="3" t="n"/>
-      <c r="S20" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T20" s="3" t="n"/>
-      <c r="U20" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V20" s="3" t="n"/>
-      <c r="W20" s="3" t="n"/>
-      <c r="X20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MF:0000008</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cognitive process</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A mental process that creates, modifies or has as participant some cognitive representation.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>mental process</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Understanding, or thinking about something or forming or changing beliefs about something. </t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Ai; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:006110</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>comprehension</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>A cognitive process that creates a representation of the meaning and significance of a communication, object, event or situation.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>cognitive process</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="n"/>
+      <c r="P21" s="3" t="n"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="n"/>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="n"/>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="n"/>
+      <c r="W21" s="3" t="n"/>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>Ai; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MFOEM:000001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>emotion process</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>An affective process that is a synchronized aggregate of constituent mental processes, including an appraisal process, which is valenced, has an object, and gives rise to an action tendency.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>mental process</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Ai; PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:013060</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>emotional BCI engagement</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Participant engagement with behaviour change intervention in which the engagement activity is an emotion process.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>emotion process</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>participant engagement with behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Engagement through having or expressing feelings or emotions in relation to an intervention. </t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Enjoying or liking the intervention</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>“Emotional BCI engagement” classes in the ontology are about how engagement is recorded or reported relevant to an individual’s response to the intervention content. Some interventions intend to elicit emotional responses as mechanisms of actions or outcomes, but these are not captured by the current class. 
+“Emotion process” is defined as “A mental process that is a synchronized aggregate of constituent mental processes including an appraisal process, which is valenced, has an object, and gives rise to an action tendency.”</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="n"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="n"/>
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V23" s="3" t="n"/>
+      <c r="W23" s="3" t="n"/>
+      <c r="X23" s="3" t="inlineStr">
         <is>
           <t>EJH; Ai; CM; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>MF:0000008</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>cognitive process</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>A mental process that creates, modifies or has as participant some cognitive representation.</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>mental process</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Understanding, or thinking about something or forming or changing beliefs about something. </t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>Ai; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:006110</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>comprehension</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>A cognitive process that creates a representation of the meaning and significance of a communication, object, event or situation.</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>cognitive process</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R22" s="3" t="n"/>
-      <c r="S22" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T22" s="3" t="n"/>
-      <c r="U22" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V22" s="3" t="n"/>
-      <c r="W22" s="3" t="n"/>
-      <c r="X22" s="3" t="inlineStr">
-        <is>
-          <t>Ai; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>MFOEM:000001</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>emotion process</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>An affective process that is a synchronized aggregate of constituent mental processes, including an appraisal process, which is valenced, has an object, and gives rise to an action tendency.</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>mental process</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Ai; PS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013060</t>
+          <t>BCIO:013065</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional BCI engagement through enjoyment</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Participant engagement with behaviour change intervention in which the engagement activity is an emotion process.</t>
+          <t xml:space="preserve">Emotional BCI engagement that involves enjoyment. </t>
         </is>
       </c>
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>emotion process</t>
+          <t>enjoyment</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>emotional BCI engagement</t>
         </is>
       </c>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engagement through having or expressing feelings or emotions in relation to an intervention. </t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Enjoying or liking the intervention</t>
-        </is>
-      </c>
+          <t>Experiencing pleasure through interacting/using the intervention (e.g., gamification).</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>“Emotional BCI engagement” classes in the ontology are about how engagement is recorded or reported relevant to an individual’s response to the intervention content. Some interventions intend to elicit emotional responses as mechanisms of actions or outcomes, but these are not captured by the current class. 
-“Emotion process” is defined as “A mental process that is a synchronized aggregate of constituent mental processes including an appraisal process, which is valenced, has an object, and gives rise to an action tendency.”</t>
+          <t>“Enjoyment” is defined as “A positive emotion that is about an ongoing experience and reflects that the experience is being appraised as pleasurable.”</t>
         </is>
       </c>
       <c r="P24" s="3" t="n"/>
@@ -2032,24 +2040,24 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013065</t>
+          <t>BCIO:050526</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through enjoyment</t>
+          <t>emotional BCI engagement through fear</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emotional BCI engagement that involves enjoyment. </t>
+          <t>Emotional BCI engagement that involves fear.</t>
         </is>
       </c>
       <c r="D25" s="3" t="n"/>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>enjoyment</t>
+          <t>fear</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2058,11 +2066,7 @@
         </is>
       </c>
       <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Experiencing pleasure through interacting/using the intervention (e.g., gamification).</t>
-        </is>
-      </c>
+      <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
@@ -2070,7 +2074,7 @@
       <c r="N25" s="3" t="n"/>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>“Enjoyment” is defined as “A positive emotion that is about an ongoing experience and reflects that the experience is being appraised as pleasurable.”</t>
+          <t>“Fear” is defined as “A negative emotion that is aversive and characterised by feelings of threat and impending doom, and by an urge to get out of the situation.”</t>
         </is>
       </c>
       <c r="P25" s="3" t="n"/>
@@ -2095,31 +2099,31 @@
       <c r="W25" s="3" t="n"/>
       <c r="X25" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; CM; PS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050526</t>
+          <t>BCIO:013075</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through fear</t>
+          <t xml:space="preserve">emotional BCI engagement through interest </t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Emotional BCI engagement that involves fear.</t>
+          <t>Emotional BCI engagement that involves interest.</t>
         </is>
       </c>
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>fear</t>
+          <t>interest</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2128,7 +2132,11 @@
         </is>
       </c>
       <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Experiencing interest in the intervention by creating a desire to learn more.</t>
+        </is>
+      </c>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
@@ -2136,7 +2144,9 @@
       <c r="N26" s="3" t="n"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>“Fear” is defined as “A negative emotion that is aversive and characterised by feelings of threat and impending doom, and by an urge to get out of the situation.”</t>
+          <t>In the Emotion Ontology, “interest” is defined as “a positive emotion which motivates learning, exploration and curiosity. Feelings of interest are associated with the novelty and complexity of stimuli.” 
+“Emotional BCI engagement through interest” can have a cognitive component or be associated with “cognitive BCI engagement through attending” or “cognitive engagement through evaluation”, as emotion and cognitive processes are often related. For instance, participants rating the “informativeness” of an intervention would qualify as a “cognitive engagement through evaluation”. 
+The opposite of interest is boredom.</t>
         </is>
       </c>
       <c r="P26" s="3" t="n"/>
@@ -2161,44 +2171,36 @@
       <c r="W26" s="3" t="n"/>
       <c r="X26" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013075</t>
+          <t>BCIO:050527</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">emotional BCI engagement through interest </t>
+          <t>emotional BCI engagement through mistrust</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Emotional BCI engagement that involves interest.</t>
+          <t xml:space="preserve">Emotional BCI engagement that involves mistrust. </t>
         </is>
       </c>
       <c r="D27" s="3" t="n"/>
       <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>interest</t>
-        </is>
-      </c>
+      <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="inlineStr">
         <is>
           <t>emotional BCI engagement</t>
         </is>
       </c>
       <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>Experiencing interest in the intervention by creating a desire to learn more.</t>
-        </is>
-      </c>
+      <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="3" t="n"/>
@@ -2206,9 +2208,7 @@
       <c r="N27" s="3" t="n"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>In the Emotion Ontology, “interest” is defined as “a positive emotion which motivates learning, exploration and curiosity. Feelings of interest are associated with the novelty and complexity of stimuli.” 
-“Emotional BCI engagement through interest” can have a cognitive component or be associated with “cognitive BCI engagement through attending” or “cognitive engagement through evaluation”, as emotion and cognitive processes are often related. For instance, participants rating the “informativeness” of an intervention would qualify as a “cognitive engagement through evaluation”. 
-The opposite of interest is boredom.</t>
+          <t>“Mistrust” is defined as “A negative emotion involving feelings of suspicion or doubt regarding the honesty, fairness, or abilities of an entity (e.g., person, object, or situation).”</t>
         </is>
       </c>
       <c r="P27" s="3" t="n"/>
@@ -2233,36 +2233,44 @@
       <c r="W27" s="3" t="n"/>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t>EJH; Ai; CM; PS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050527</t>
+          <t>BCIO:013070</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through mistrust</t>
+          <t xml:space="preserve">emotional BCI engagement through satisfaction </t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emotional BCI engagement that involves mistrust. </t>
+          <t>Emotional BCI engagement that involves satisfaction.</t>
         </is>
       </c>
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>satisfaction</t>
+        </is>
+      </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
           <t>emotional BCI engagement</t>
         </is>
       </c>
       <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Experiencing satisfaction by fulfilling needs, expectations or wishes. </t>
+        </is>
+      </c>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="n"/>
       <c r="L28" s="3" t="n"/>
@@ -2270,7 +2278,7 @@
       <c r="N28" s="3" t="n"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>“Mistrust” is defined as “A negative emotion involving feelings of suspicion or doubt regarding the honesty, fairness, or abilities of an entity (e.g., person, object, or situation).”</t>
+          <t>“Satisfaction” is defined as “An emotion that is experienced when one's wishes, expectations or needs are fulfilled.”</t>
         </is>
       </c>
       <c r="P28" s="3" t="n"/>
@@ -2295,94 +2303,66 @@
       <c r="W28" s="3" t="n"/>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:013070</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">emotional BCI engagement through satisfaction </t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Emotional BCI engagement that involves satisfaction.</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>satisfaction</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>emotional BCI engagement</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Experiencing satisfaction by fulfilling needs, expectations or wishes. </t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>“Satisfaction” is defined as “An emotion that is experienced when one's wishes, expectations or needs are fulfilled.”</t>
-        </is>
-      </c>
-      <c r="P29" s="3" t="n"/>
-      <c r="Q29" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R29" s="3" t="n"/>
-      <c r="S29" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T29" s="3" t="n"/>
-      <c r="U29" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V29" s="3" t="n"/>
-      <c r="W29" s="3" t="n"/>
-      <c r="X29" s="3" t="inlineStr">
-        <is>
-          <t>EJH; Ai; CM; PS</t>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MFOEM:000218</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>enjoyment</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A positive emotion that is about an ongoing experience and reflects that the experience is being appraised as pleasurable</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>emotion process</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Ai</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MFOEM:000218</t>
+          <t>MFOEM:000026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>enjoyment</t>
+          <t>fear</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>A positive emotion that is about an ongoing experience and reflects that the experience is being appraised as pleasurable</t>
+          <t>A negative emotion that is aversive and characterised by feelings of threat and impending doom, and by an urge to get out of the situation.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2390,11 +2370,6 @@
           <t>emotion process</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
       <c r="S30" t="inlineStr">
         <is>
           <t>0</t>
@@ -2403,28 +2378,23 @@
       <c r="U30" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>Ai</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MFOEM:000026</t>
+          <t>MFOEM:000033</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>fear</t>
+          <t>interest</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A negative emotion that is aversive and characterised by feelings of threat and impending doom, and by an urge to get out of the situation.</t>
+          <t>Interest is a positive emotion which motivates learning, exploration and curiosity. Feelings of interest are associated with the novelty and complexity of stimuli</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2432,6 +2402,11 @@
           <t>emotion process</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
       <c r="S31" t="inlineStr">
         <is>
           <t>0</t>
@@ -2442,46 +2417,71 @@
           <t>External</t>
         </is>
       </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Ai</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>MFOEM:000033</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>interest</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Interest is a positive emotion which motivates learning, exploration and curiosity. Feelings of interest are associated with the novelty and complexity of stimuli</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>emotion process</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>Ai</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050521</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>intervention engagement period statistic</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>A data item that is about a collection of intervention engagement periods.</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>BCI engagement period</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="n"/>
+      <c r="N32" s="3" t="n"/>
+      <c r="O32" s="3" t="n"/>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="n"/>
+      <c r="U32" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V32" s="3" t="n"/>
+      <c r="W32" s="3" t="n"/>
+      <c r="X32" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
         </is>
       </c>
     </row>
@@ -2530,36 +2530,36 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050528</t>
+          <t>BCIO:050529</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>maximum BCI engagement period</t>
+          <t>maximum aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>A BCI engagement period statistic that is the highest value from a collection of BCI engagement periods.</t>
+          <t>An aggregate behavioural BCI engagement duration statistic that is the highest value from a collection of aggregate behavioural BCI engagement durations.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period statistic</t>
+          <t>aggregate behavioural BCI engagement duration statistic</t>
         </is>
       </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>The maximum period of intervention that participants engaged with.</t>
+          <t>The maximum duration of all intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K34" s="3" t="n"/>
@@ -2596,36 +2596,36 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050529</t>
+          <t>BCIO:050531</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>maximum aggregate behavioural BCI engagement duration</t>
+          <t>maximum behavioural BCI engagement frequency</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>An aggregate behavioural BCI engagement duration statistic that is the highest value from a collection of aggregate behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement frequency statistic that is the highest value from a collection of behavioural BCI engagement frequencies.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement frequency statistic</t>
         </is>
       </c>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>The maximum duration of all intervention sessions attended by participants.</t>
+          <t>The maximum frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K35" s="3" t="n"/>
@@ -2662,36 +2662,36 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050530</t>
+          <t>BCIO:050532</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural BCI engagement duration</t>
+          <t>maximum behavioural BCI engagement number</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement duration statistic that is the highest value from a collection of behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement number statistic that is the highest value from a collection of behavioural BCI engagement numbers.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement number statistic</t>
         </is>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>The maximum duration of intervention sessions attended by participants.</t>
+          <t>The maximum number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K36" s="3" t="n"/>
@@ -2728,36 +2728,36 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050531</t>
+          <t>BCIO:050530</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural BCI engagement frequency</t>
+          <t>maximum behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the highest value from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the highest value from a collection of behavioural intervention| engagement durations.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>The maximum frequency of intervention sessions attended by participants.</t>
+          <t>The maximum duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K37" s="3" t="n"/>
@@ -2794,36 +2794,36 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050532</t>
+          <t>BCIO:050528</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural BCI engagement number</t>
+          <t>maximum intervention engagement period</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the highest value from a collection of behavioural BCI engagement numbers.</t>
+          <t>An intervention engagement period statistic that is the highest value from a collection of intervention engagement periods.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>BCI engagement period</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>intervention engagement period statistic</t>
         </is>
       </c>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>The maximum number of intervention sessions attended by participants.</t>
+          <t>The maximum period of intervention that participants engaged with.</t>
         </is>
       </c>
       <c r="K38" s="3" t="n"/>
@@ -2860,36 +2860,36 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050533</t>
+          <t>BCIO:050534</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>mean BCI engagement period</t>
+          <t>mean aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>A BCI engagement period statistic that is the average value calculated from a collection of BCI engagement periods.</t>
+          <t>An aggregate behavioural BCI engagement duration statistic that is the average value calculated from a collection of aggregate behavioural BCI engagement durations.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period statistic</t>
+          <t>aggregate behavioural BCI engagement duration statistic</t>
         </is>
       </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>The mean period of intervention  that participants engaged with.</t>
+          <t>The mean duration of all intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K39" s="3" t="n"/>
@@ -2926,36 +2926,36 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050534</t>
+          <t>BCIO:050536</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>mean aggregate behavioural BCI engagement duration</t>
+          <t>mean behavioural BCI engagement frequency</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>An aggregate behavioural BCI engagement duration statistic that is the average value calculated from a collection of aggregate behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement frequency statistic that is the average value calculated from a collection of behavioural BCI engagement frequencies.</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement frequency statistic</t>
         </is>
       </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>The mean duration of all intervention sessions attended by participants.</t>
+          <t>The mean frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K40" s="3" t="n"/>
@@ -2992,36 +2992,36 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050535</t>
+          <t>BCIO:050537</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural BCI engagement duration</t>
+          <t>mean behavioural BCI engagement number</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement duration statistic that is the average value calculated from a collection of behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement number statistic that is the average value calculated from a collection of behavioural BCI engagement numbers.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement number statistic</t>
         </is>
       </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>The mean duration of intervention sessions attended by participants.</t>
+          <t>The mean number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K41" s="3" t="n"/>
@@ -3058,36 +3058,36 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050536</t>
+          <t>BCIO:050535</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural BCI engagement frequency</t>
+          <t>mean behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the average value calculated from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the average value calculated from a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>The mean frequency of intervention sessions attended by participants.</t>
+          <t>The mean duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K42" s="3" t="n"/>
@@ -3124,36 +3124,36 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050537</t>
+          <t>BCIO:050533</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural BCI engagement number</t>
+          <t>mean intervention engagement period</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the average value calculated from a collection of behavioural BCI engagement numbers.</t>
+          <t>An intervention engagement period statistic that is the average value calculated from a collection of intervention engagement periods.</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>BCI engagement period</t>
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>intervention engagement period statistic</t>
         </is>
       </c>
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>The mean number of intervention sessions attended by participants.</t>
+          <t>The mean period of intervention  that participants engaged with.</t>
         </is>
       </c>
       <c r="K43" s="3" t="n"/>
@@ -3190,36 +3190,36 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050538</t>
+          <t>BCIO:050539</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>median BCI engagement period</t>
+          <t>median aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>A BCI engagement period statistic that is the central value of a collection of BCI engagement periods.</t>
+          <t>An aggregate behavioural BCI engagement duration statistic that is the central value of a collection of aggregate behavioural BCI engagement durations.</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period statistic</t>
+          <t>aggregate behavioural BCI engagement duration statistic</t>
         </is>
       </c>
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>The median period of intervention that participants engaged with.</t>
+          <t>The median duration of all intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K44" s="3" t="n"/>
@@ -3256,36 +3256,36 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050539</t>
+          <t>BCIO:050541</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>median aggregate behavioural BCI engagement duration</t>
+          <t>median behavioural BCI engagement frequency</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>An aggregate behavioural BCI engagement duration statistic that is the central value of a collection of aggregate behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement frequency statistic that is the central value of a collection of behavioural BCI engagement frequencies.</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement frequency statistic</t>
         </is>
       </c>
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>The median duration of all intervention sessions attended by participants.</t>
+          <t>The median frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K45" s="3" t="n"/>
@@ -3322,36 +3322,36 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050540</t>
+          <t>BCIO:050542</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>median behavioural BCI engagement duration</t>
+          <t>median behavioural BCI engagement number</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement duration statistic that is the central value of a collection of behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement number statistic that is the central value of a collection of behavioural BCI engagement numbers.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement number statistic</t>
         </is>
       </c>
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>The median duration of intervention sessions attended by participants.</t>
+          <t>The median number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K46" s="3" t="n"/>
@@ -3388,36 +3388,36 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050541</t>
+          <t>BCIO:050540</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>median behavioural BCI engagement frequency</t>
+          <t>median behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the central value of a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the central value of a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>The median frequency of intervention sessions attended by participants.</t>
+          <t>The median duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K47" s="3" t="n"/>
@@ -3454,36 +3454,36 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050542</t>
+          <t>BCIO:050538</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>median behavioural BCI engagement number</t>
+          <t>median intervention engagement period</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the central value of a collection of behavioural BCI engagement numbers.</t>
+          <t>An intervention engagement period statistic that is the central value of a collection of intervention engagement periods.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>BCI engagement period</t>
         </is>
       </c>
       <c r="E48" s="3" t="n"/>
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>intervention engagement period statistic</t>
         </is>
       </c>
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>The median number of intervention sessions attended by participants.</t>
+          <t>The median period of intervention that participants engaged with.</t>
         </is>
       </c>
       <c r="K48" s="3" t="n"/>
@@ -3520,36 +3520,36 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050543</t>
+          <t>BCIO:050544</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>minimum BCI engagement period</t>
+          <t>minimum aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>A BCI engagement period statistic that is the lowest value from a collection of BCI engagement periods.</t>
+          <t>An aggregate behavioural BCI engagement duration statistic that is the lowest value from a collection of aggregate behavioural BCI engagement durations.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>aggregate behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E49" s="3" t="n"/>
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period statistic</t>
+          <t>aggregate behavioural BCI engagement duration statistic</t>
         </is>
       </c>
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>The minimum period of intervention that participants engaged with.</t>
+          <t>The minimum duration of all intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K49" s="3" t="n"/>
@@ -3586,36 +3586,36 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050544</t>
+          <t>BCIO:050546</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>minimum aggregate behavioural BCI engagement duration</t>
+          <t>minimum behavioural BCI engagement frequency</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>An aggregate behavioural BCI engagement duration statistic that is the lowest value from a collection of aggregate behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement frequency statistic that is the lowest value from a collection of behavioural BCI engagement frequencies.</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement frequency statistic</t>
         </is>
       </c>
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>The minimum duration of all intervention sessions attended by participants.</t>
+          <t>The minimum frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K50" s="3" t="n"/>
@@ -3652,36 +3652,36 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050545</t>
+          <t>BCIO:050547</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural BCI engagement duration</t>
+          <t>minimum behavioural BCI engagement number</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement duration statistic that is the lowest value from a collection of behavioural BCI engagement durations.</t>
+          <t>A behavioural BCI engagement number statistic that is the lowest value from a collection of behavioural BCI engagement numbers.</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E51" s="3" t="n"/>
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration statistic</t>
+          <t>behavioural BCI engagement number statistic</t>
         </is>
       </c>
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>The minimum duration of intervention sessions attended by participants.</t>
+          <t>The minimum number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K51" s="3" t="n"/>
@@ -3718,36 +3718,36 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050546</t>
+          <t>BCIO:050545</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural BCI engagement frequency</t>
+          <t>minimum behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the lowest value from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the lowest value from a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>The minimum frequency of intervention sessions attended by participants.</t>
+          <t>The minimum duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K52" s="3" t="n"/>
@@ -3784,36 +3784,36 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050547</t>
+          <t>BCIO:050543</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural BCI engagement number</t>
+          <t>minimum intervention engagement period</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the lowest value from a collection of behavioural BCI engagement numbers.</t>
+          <t>An intervention engagement period statistic that is the lowest value from a collection of intervention engagement periods.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>BCI engagement period</t>
         </is>
       </c>
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3" t="n"/>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>intervention engagement period statistic</t>
         </is>
       </c>
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>The minimum number of intervention sessions attended by participants.</t>
+          <t>The minimum period of intervention that participants engaged with.</t>
         </is>
       </c>
       <c r="K53" s="3" t="n"/>

</xml_diff>

<commit_message>
Update 12 terms in BCIO_Engagement.xlsx
</commit_message>
<xml_diff>
--- a/Engagement/BCIO_Engagement.xlsx
+++ b/Engagement/BCIO_Engagement.xlsx
@@ -1202,22 +1202,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013020</t>
+          <t>BCIO:050523</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about the number of times behavioural BCI engagement occurs within a unit of time.</t>
+          <t>A data item that is about a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E12" s="3" t="n"/>
@@ -1229,88 +1229,88 @@
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hourly, daily, weekly or monthly encounters. </t>
-        </is>
-      </c>
+      <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="n"/>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="n"/>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="n"/>
+      <c r="W12" s="3" t="n"/>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:013020</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>behavioural intervention engagement frequency</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>A data item that is about the number of times behavioural intervention engagement occurs within a unit of time.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>behavioural BCI engagement</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hourly, daily, weekly or monthly encounters. </t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median</t>
         </is>
       </c>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Describes the frequency of BCI engagement in a BCI (e.g., participants had weekly contact), or the frequency of engagement in part of a BCI (e.g., participants received face-to-face contact once a month). 
 The class “BCI engagement frequency” can be used to capture the frequency of different types of engagement, such as the frequency of engaging with social media or printed material. 
 Depending on how “BCI engagement frequency” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants joined at least 1 session every week), (2) maximum (e.g., only 10% of participants attended 5 sessions every week), (3) mean (e.g., participants joined 4 sessions per week on average) or (4) median (e.g., the median number of sessions participants attended was 4 per week). </t>
         </is>
       </c>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="n"/>
-      <c r="U12" s="3" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V12" s="3" t="n"/>
-      <c r="W12" s="3" t="n"/>
-      <c r="X12" s="3" t="inlineStr">
-        <is>
-          <t>EJH; Ai; CM; PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050524</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>behavioural BCI engagement frequency statistic</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>A data item that is about a collection of behavioural BCI engagement frequencies.</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>behavioural BCI engagement</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
       <c r="P13" s="3" t="n"/>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -1333,24 +1333,24 @@
       <c r="W13" s="3" t="n"/>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>EJH; Ai; CM; PS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050525</t>
+          <t>BCIO:050524</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>behavioural intervention engagement frequency statistic</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about a collection of behavioural BCI engagement contact event numbers.</t>
+          <t>A data item that is about a collection of behavioural intervention engagement frequencies.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1402,22 +1402,22 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050523</t>
+          <t>BCIO:050525</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>behavioural intervention engagement duration statistic</t>
+          <t>behavioural intervention engagement number statistic</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about a collection of behavioural intervention engagement durations.</t>
+          <t>A data item that is about a collection of behavioural intervention engagement contact event numbers.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E15" s="3" t="n"/>
@@ -2596,36 +2596,36 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050531</t>
+          <t>BCIO:050530</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural BCI engagement frequency</t>
+          <t>maximum behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the highest value from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the highest value from a collection of behavioural intervention| engagement durations.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>The maximum frequency of intervention sessions attended by participants.</t>
+          <t>The maximum duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K35" s="3" t="n"/>
@@ -2662,17 +2662,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050532</t>
+          <t>BCIO:050531</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural BCI engagement number</t>
+          <t>maximum behavioural intervention engagement frequency</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the highest value from a collection of behavioural BCI engagement numbers.</t>
+          <t>A behavioural intervention engagement frequency statistic that is the highest value from a collection of behavioural intervention engagement frequencies.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2684,14 +2684,14 @@
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>behavioural intervention engagement frequency statistic</t>
         </is>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>The maximum number of intervention sessions attended by participants.</t>
+          <t>The maximum frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K36" s="3" t="n"/>
@@ -2728,36 +2728,36 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050530</t>
+          <t>BCIO:050532</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>maximum behavioural intervention engagement duration</t>
+          <t>maximum behavioural intervention engagement number</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>A behavioural intervention engagement duration statistic that is the highest value from a collection of behavioural intervention| engagement durations.</t>
+          <t>A behavioural intervention engagement number statistic that is the highest value from a collection of behavioural intervention engagement numbers.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>behavioural intervention engagement duration statistic</t>
+          <t>behavioural intervention engagement number statistic</t>
         </is>
       </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>The maximum duration of intervention sessions attended by participants.</t>
+          <t>The maximum number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K37" s="3" t="n"/>
@@ -2926,36 +2926,36 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050536</t>
+          <t>BCIO:050535</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural BCI engagement frequency</t>
+          <t>mean behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the average value calculated from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the average value calculated from a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>The mean frequency of intervention sessions attended by participants.</t>
+          <t>The mean duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K40" s="3" t="n"/>
@@ -2992,17 +2992,17 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050537</t>
+          <t>BCIO:050536</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural BCI engagement number</t>
+          <t>mean behavioural intervention engagement frequency</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the average value calculated from a collection of behavioural BCI engagement numbers.</t>
+          <t>A behavioural intervention engagement frequency statistic that is the average value calculated from a collection of behavioural intervention engagement frequencies.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -3014,14 +3014,14 @@
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>behavioural intervention engagement frequency statistic</t>
         </is>
       </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>The mean number of intervention sessions attended by participants.</t>
+          <t>The mean frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K41" s="3" t="n"/>
@@ -3058,36 +3058,36 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050535</t>
+          <t>BCIO:050537</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>mean behavioural intervention engagement duration</t>
+          <t>mean behavioural intervention engagement number</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>A behavioural intervention engagement duration statistic that is the average value calculated from a collection of behavioural intervention engagement durations.</t>
+          <t>A behavioural intervention engagement number statistic that is the average value calculated from a collection of behavioural intervention engagement numbers.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>behavioural intervention engagement duration statistic</t>
+          <t>behavioural intervention engagement number statistic</t>
         </is>
       </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>The mean duration of intervention sessions attended by participants.</t>
+          <t>The mean number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K42" s="3" t="n"/>
@@ -3256,36 +3256,36 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050541</t>
+          <t>BCIO:050540</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>median behavioural BCI engagement frequency</t>
+          <t>median behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the central value of a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the central value of a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>The median frequency of intervention sessions attended by participants.</t>
+          <t>The median duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K45" s="3" t="n"/>
@@ -3322,17 +3322,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050542</t>
+          <t>BCIO:050541</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>median behavioural BCI engagement number</t>
+          <t>median behavioural intervention engagement frequency</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the central value of a collection of behavioural BCI engagement numbers.</t>
+          <t>A behavioural intervention engagement frequency statistic that is the central value of a collection of behavioural intervention engagement frequencies.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3344,14 +3344,14 @@
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>behavioural intervention engagement frequency statistic</t>
         </is>
       </c>
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>The median number of intervention sessions attended by participants.</t>
+          <t>The median frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K46" s="3" t="n"/>
@@ -3388,36 +3388,36 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050540</t>
+          <t>BCIO:050542</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>median behavioural intervention engagement duration</t>
+          <t>median behavioural intervention engagement number</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>A behavioural intervention engagement duration statistic that is the central value of a collection of behavioural intervention engagement durations.</t>
+          <t>A behavioural intervention engagement number statistic that is the central value of a collection of behavioural intervention engagement numbers.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>behavioural intervention engagement duration statistic</t>
+          <t>behavioural intervention engagement number statistic</t>
         </is>
       </c>
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>The median duration of intervention sessions attended by participants.</t>
+          <t>The median number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K47" s="3" t="n"/>
@@ -3586,36 +3586,36 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050546</t>
+          <t>BCIO:050545</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural BCI engagement frequency</t>
+          <t>minimum behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement frequency statistic that is the lowest value from a collection of behavioural BCI engagement frequencies.</t>
+          <t>A behavioural intervention engagement duration statistic that is the lowest value from a collection of behavioural intervention engagement durations.</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural BCI engagement duration</t>
         </is>
       </c>
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement frequency statistic</t>
+          <t>behavioural intervention engagement duration statistic</t>
         </is>
       </c>
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>The minimum frequency of intervention sessions attended by participants.</t>
+          <t>The minimum duration of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K50" s="3" t="n"/>
@@ -3652,17 +3652,17 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050547</t>
+          <t>BCIO:050546</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural BCI engagement number</t>
+          <t>minimum behavioural intervention engagement frequency</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>A behavioural BCI engagement number statistic that is the lowest value from a collection of behavioural BCI engagement numbers.</t>
+          <t>A behavioural intervention engagement frequency statistic that is the lowest value from a collection of behavioural intervention engagement frequencies.</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3674,14 +3674,14 @@
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement number statistic</t>
+          <t>behavioural intervention engagement frequency statistic</t>
         </is>
       </c>
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>The minimum number of intervention sessions attended by participants.</t>
+          <t>The minimum frequency of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K51" s="3" t="n"/>
@@ -3718,36 +3718,36 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050545</t>
+          <t>BCIO:050547</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>minimum behavioural intervention engagement duration</t>
+          <t>minimum behavioural intervention engagement number</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>A behavioural intervention engagement duration statistic that is the lowest value from a collection of behavioural intervention engagement durations.</t>
+          <t>A behavioural intervention engagement number statistic that is the lowest value from a collection of behavioural intervention engagement numbers.</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural BCI engagement</t>
         </is>
       </c>
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>behavioural intervention engagement duration statistic</t>
+          <t>behavioural intervention engagement number statistic</t>
         </is>
       </c>
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>The minimum duration of intervention sessions attended by participants.</t>
+          <t>The minimum number of intervention sessions attended by participants.</t>
         </is>
       </c>
       <c r="K52" s="3" t="n"/>
@@ -3897,12 +3897,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>number of behavioural BCI engagements</t>
+          <t>number of behavioural intervention engagements</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about the number of times behavioural BCI engagement occurs.</t>
+          <t>A data item that is about the number of times behavioural intervention engagement occurs.</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update 11 terms in BCIO_Engagement.xlsx
</commit_message>
<xml_diff>
--- a/Engagement/BCIO_Engagement.xlsx
+++ b/Engagement/BCIO_Engagement.xlsx
@@ -1053,45 +1053,54 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013010</t>
+          <t>BCIO:013025</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
+          <t>behavioural BCI engagement duration</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal interval between the start and end of a behavioural BCI engagement. </t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
           <t>behavioural BCI engagement</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Participant engagement with behaviour change intervention in which the engagement activity is a behaviour. </t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>one-dimensional temporal region</t>
         </is>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Any behaviour performed to engage with an intervention and its content.</t>
+          <t>A unit of time that describes the length of an engagement event.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Eye movements, body movements, meditation, attending an intervention session, using nicotine patches in a smoking cessation intervention, or online activity: attending, logging in, posting on a discussion board, reading content, mouse clicks, viewing, using tools, journaling</t>
+          <t>A 30-minute session, 1 hour spent 'logged in'</t>
         </is>
       </c>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median</t>
+        </is>
+      </c>
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>This is distinguished from engagement that involves thought processes.</t>
+          <t>The class “BCI engagement duration” can be used multiple times to capture the frequency of different types of engagements, such as the frequency of engaging with social media or printed material. 
+Depending on how “BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 10 minutes in each session, (2) maximum (e.g., participants talked to the therapist for up to 1 hour in each session, (3) mean (e.g., participants talked with the therapist for 45 minutes on average in each session) or (4) median (e.g., the median length of calls between participants and therapists was 42 minutes in each session).</t>
         </is>
       </c>
       <c r="P10" s="3" t="n"/>
@@ -1123,54 +1132,45 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BCIO:013025</t>
+          <t>BCIO:013010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A temporal interval between the start and end of a behavioural BCI engagement. </t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>behavioural BCI engagement</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Participant engagement with  intervention in which the engagement activity is a behaviour. </t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>A unit of time that describes the length of an engagement event.</t>
+          <t>Any behaviour performed to engage with an intervention and its content.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>A 30-minute session, 1 hour spent 'logged in'</t>
+          <t>Eye movements, body movements, meditation, attending an intervention session, using nicotine patches in a smoking cessation intervention, or online activity: attending, logging in, posting on a discussion board, reading content, mouse clicks, viewing, using tools, journaling</t>
         </is>
       </c>
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Mean;Minimum;Maximum;Median</t>
-        </is>
-      </c>
+      <c r="M11" s="3" t="n"/>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>The class “BCI engagement duration” can be used multiple times to capture the frequency of different types of engagements, such as the frequency of engaging with social media or printed material. 
-Depending on how “BCI engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 10 minutes in each session, (2) maximum (e.g., participants talked to the therapist for up to 1 hour in each session, (3) mean (e.g., participants talked with the therapist for 45 minutes on average in each session) or (4) median (e.g., the median length of calls between participants and therapists was 42 minutes in each session).</t>
+          <t>This is distinguished from engagement that involves thought processes.</t>
         </is>
       </c>
       <c r="P11" s="3" t="n"/>
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement</t>
+          <t>cognitive intervention engagement</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Participant engagement with behaviour change intervention in which the engagement activity is a cognitive process.</t>
+          <t>Participant engagement with intervention in which the engagement activity is a cognitive process.</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="H16" s="3" t="n"/>
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cognitive BCI engagement through attention </t>
+          <t xml:space="preserve">cognitive intervention engagement through attention </t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>A cognitive BCI engagement that involves attending.</t>
+          <t>A cognitive intervention engagement that involves attending.</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement</t>
+          <t>cognitive intervention engagement</t>
         </is>
       </c>
       <c r="H17" s="3" t="n"/>
@@ -1613,12 +1613,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cognitive BCI engagement through comprehension </t>
+          <t xml:space="preserve">cognitive intervention engagement through comprehension </t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>A cognitive BCI engagement that involves comprehension.</t>
+          <t>A cognitive intervention engagement that involves comprehension.</t>
         </is>
       </c>
       <c r="D18" s="3" t="n"/>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement</t>
+          <t>cognitive intervention engagement</t>
         </is>
       </c>
       <c r="H18" s="3" t="n"/>
@@ -1683,12 +1683,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement through judging</t>
+          <t>cognitive intervention engagement through judging</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>A cognitive BCI engagement that involves a judging process.</t>
+          <t>A cognitive intervention engagement that involves a judging process.</t>
         </is>
       </c>
       <c r="D19" s="3" t="n"/>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>cognitive BCI engagement</t>
+          <t>cognitive intervention engagement</t>
         </is>
       </c>
       <c r="H19" s="3" t="n"/>
@@ -1900,12 +1900,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional intervention engagement</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Participant engagement with behaviour change intervention in which the engagement activity is an emotion process.</t>
+          <t>Participant engagement with intervention in which the engagement activity is an emotion process.</t>
         </is>
       </c>
       <c r="D23" s="3" t="n"/>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="H23" s="3" t="n"/>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through enjoyment</t>
+          <t>emotional intervention engagement through enjoyment</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emotional BCI engagement that involves enjoyment. </t>
+          <t xml:space="preserve">Emotional intervention engagement that involves enjoyment. </t>
         </is>
       </c>
       <c r="D24" s="3" t="n"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional intervention engagement</t>
         </is>
       </c>
       <c r="H24" s="3" t="n"/>
@@ -2045,12 +2045,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through fear</t>
+          <t>emotional intervention engagement through fear</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Emotional BCI engagement that involves fear.</t>
+          <t>Emotional intervention engagement that involves fear.</t>
         </is>
       </c>
       <c r="D25" s="3" t="n"/>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional intervention engagement</t>
         </is>
       </c>
       <c r="H25" s="3" t="n"/>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">emotional BCI engagement through interest </t>
+          <t xml:space="preserve">emotional intervention engagement through interest </t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Emotional BCI engagement that involves interest.</t>
+          <t>Emotional intervention engagement that involves interest.</t>
         </is>
       </c>
       <c r="D26" s="3" t="n"/>
@@ -2128,10 +2128,10 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="n"/>
+          <t>emotioenal BI engge</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Experiencing interest in the intervention by creating a desire to learn more.</t>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement through mistrust</t>
+          <t>emotional intervention engagement through mistrust</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emotional BCI engagement that involves mistrust. </t>
+          <t xml:space="preserve">Emotional intervention engagement that involves mistrust. </t>
         </is>
       </c>
       <c r="D27" s="3" t="n"/>
@@ -2196,7 +2196,7 @@
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional intervention engagement</t>
         </is>
       </c>
       <c r="H27" s="3" t="n"/>
@@ -2245,12 +2245,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">emotional BCI engagement through satisfaction </t>
+          <t xml:space="preserve">emotional intervention engagement through satisfaction </t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Emotional BCI engagement that involves satisfaction.</t>
+          <t>Emotional intervention engagement that involves satisfaction.</t>
         </is>
       </c>
       <c r="D28" s="3" t="n"/>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>emotional BCI engagement</t>
+          <t>emotional intervention engagement</t>
         </is>
       </c>
       <c r="H28" s="3" t="n"/>

</xml_diff>

<commit_message>
Update 20 terms in BCIO_Engagement.xlsx
</commit_message>
<xml_diff>
--- a/Engagement/BCIO_Engagement.xlsx
+++ b/Engagement/BCIO_Engagement.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="E11" s="3" t="n"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E14" s="3" t="n"/>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E31" s="3" t="n"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>intervention engagement period</t>
         </is>
       </c>
       <c r="E32" s="3" t="n"/>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="E35" s="3" t="n"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>intervention engagement period</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>intervention engagement period</t>
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E46" s="3" t="n"/>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>intervention engagement period</t>
         </is>
       </c>
       <c r="E48" s="3" t="n"/>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement duration</t>
         </is>
       </c>
       <c r="E50" s="3" t="n"/>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E51" s="3" t="n"/>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>behavioural BCI engagement</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E52" s="3" t="n"/>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>BCI engagement period</t>
+          <t>intervention engagement period</t>
         </is>
       </c>
       <c r="E53" s="3" t="n"/>

</xml_diff>

<commit_message>
Update 5 terms in BCIO_Engagement.xlsx
</commit_message>
<xml_diff>
--- a/Engagement/BCIO_Engagement.xlsx
+++ b/Engagement/BCIO_Engagement.xlsx
@@ -881,7 +881,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>aggregate behavioural BCI engagement duration</t>
+          <t>behavioural intervention engagement</t>
         </is>
       </c>
       <c r="E7" s="3" t="n"/>
@@ -892,13 +892,27 @@
         </is>
       </c>
       <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>A unit of time that describes the summed duration of all intervention engagement events.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>90 minutes total app usage, 12 hours of counselling sessions</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>"Describes the total duration of engagement in an intervention (e.g., all face-to-face sessions AND all telephone contacts), or the total duration of engagement in part of an intervention (e.g., all face-to-face sessions only). (A unit of time that describes the summed duration of all intervention engagement events.) 
+Depending on how “aggregate intervention engagement duration” is reported in interventions, it can be annotated with different data items, e.g. (1) minimum (e.g., all participants talked to the therapist for at least 50 minutes in total across the sessions, (2) maximum (e.g., participants talked to the therapist for up to 4.5 hours in total across the sessions, (3) mean (e.g., participants talked with the therapist, on average, for 3 hours in total across the sessions) or (4) median (e.g., the median length of time participants talked with therapists in all their session was 3 hours)."
+This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
       <c r="P7" s="3" t="n"/>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -2573,11 +2587,7 @@
           <t>An aggregate behavioural intervention engagement duration that is the highest value from a collection of aggregate behavioural intervention engagement durations.</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
+      <c r="D34" s="3" t="inlineStr"/>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="inlineStr">
@@ -2923,11 +2933,7 @@
           <t>An aggregate behavioural intervention engagement duration that is the average value calculated from a collection of aggregate behavioural intervention engagement durations.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
+      <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="inlineStr">
@@ -3273,11 +3279,7 @@
           <t>An aggregate behavioural intervention engagement duration that is the central value of a collection of aggregate behavioural intervention engagement durations.</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
+      <c r="D44" s="3" t="inlineStr"/>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="inlineStr">
@@ -3623,12 +3625,8 @@
           <t>An aggregate behavioural intervention engagement duration that is the lowest value from a collection of aggregate behavioural intervention engagement durations.</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>aggregate behavioural BCI engagement duration</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="n"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="inlineStr">
         <is>

</xml_diff>